<commit_message>
login system updated with using  OOPS Concept
</commit_message>
<xml_diff>
--- a/Users.xlsx
+++ b/Users.xlsx
@@ -73,13 +73,13 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="FFBFBFBF"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FFBFBFBF"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -93,7 +93,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A1B1D"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>

</xml_diff>